<commit_message>
Fix Intake Column type
</commit_message>
<xml_diff>
--- a/student application tracker.xlsx
+++ b/student application tracker.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="161">
   <si>
     <t>Student ID</t>
   </si>
@@ -492,6 +492,24 @@
   </si>
   <si>
     <t>This is a prototype built with fictional sample data. All names, IDs, dates and staff are made up. It contains no real student or company information.</t>
+  </si>
+  <si>
+    <t>Angola</t>
+  </si>
+  <si>
+    <t>MSc Artificial Intelligence</t>
+  </si>
+  <si>
+    <t>Trinity College</t>
+  </si>
+  <si>
+    <t>Jan 2026</t>
+  </si>
+  <si>
+    <t>Sep 2026</t>
+  </si>
+  <si>
+    <t>Sep 2027</t>
   </si>
 </sst>
 </file>
@@ -549,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -558,9 +576,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -951,7 +972,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>153</v>
       </c>
     </row>
@@ -974,7 +995,7 @@
     <col min="1" max="4" width="14.6328125" customWidth="1"/>
     <col min="5" max="5" width="38.6328125" customWidth="1"/>
     <col min="6" max="6" width="28.6328125" customWidth="1"/>
-    <col min="7" max="7" width="14.6328125" customWidth="1"/>
+    <col min="7" max="7" width="14.6328125" style="6" customWidth="1"/>
     <col min="8" max="8" width="14.6328125" style="3" customWidth="1"/>
     <col min="9" max="10" width="14.6328125" customWidth="1"/>
     <col min="11" max="11" width="30.6328125" customWidth="1"/>
@@ -1001,7 +1022,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
@@ -1039,6 +1060,21 @@
       <c r="B2" t="s">
         <v>27</v>
       </c>
+      <c r="C2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>158</v>
+      </c>
       <c r="I2" t="s">
         <v>18</v>
       </c>
@@ -1053,6 +1089,9 @@
         <f ca="1">IF(A2="","",IF(OR(I2="Arrived",I2="Withdrawn"),"Closed",IF(M2="","No deadline",IF(M2&lt;0,"Overdue",IF(M2&lt;=7,"Due this week",IF(M2&lt;=14,"Due soon","On track"))))))</f>
         <v>Overdue</v>
       </c>
+      <c r="O2" t="s">
+        <v>149</v>
+      </c>
       <c r="P2">
         <f ca="1">IF(OR(N2="Overdue",N2="Due this week"),COUNTIF(N$2:N2,"Overdue")+COUNTIF(N$2:N2,"Due this week"),"")</f>
         <v>1</v>
@@ -1077,8 +1116,8 @@
       <c r="F3" t="s">
         <v>34</v>
       </c>
-      <c r="G3" t="s">
-        <v>35</v>
+      <c r="G3" s="6" t="s">
+        <v>159</v>
       </c>
       <c r="H3" s="3">
         <v>46056</v>
@@ -1124,7 +1163,7 @@
       <c r="F4" t="s">
         <v>34</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H4" s="3">
@@ -1174,7 +1213,7 @@
       <c r="F5" t="s">
         <v>41</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H5" s="3">
@@ -1224,7 +1263,7 @@
       <c r="F6" t="s">
         <v>45</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H6" s="3">
@@ -1277,7 +1316,7 @@
       <c r="F7" t="s">
         <v>41</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H7" s="3">
@@ -1330,7 +1369,7 @@
       <c r="F8" t="s">
         <v>41</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H8" s="3">
@@ -1383,7 +1422,7 @@
       <c r="F9" t="s">
         <v>41</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H9" s="3">
@@ -1436,7 +1475,7 @@
       <c r="F10" t="s">
         <v>56</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H10" s="3">
@@ -1489,7 +1528,7 @@
       <c r="F11" t="s">
         <v>45</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H11" s="3">
@@ -1539,7 +1578,7 @@
       <c r="F12" t="s">
         <v>62</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H12" s="3">
@@ -1592,7 +1631,7 @@
       <c r="F13" t="s">
         <v>41</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H13" s="3">
@@ -1645,7 +1684,7 @@
       <c r="F14" t="s">
         <v>41</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H14" s="3">
@@ -1698,7 +1737,7 @@
       <c r="F15" t="s">
         <v>34</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H15" s="3">
@@ -1751,7 +1790,7 @@
       <c r="F16" t="s">
         <v>56</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H16" s="3">
@@ -1804,7 +1843,7 @@
       <c r="F17" t="s">
         <v>56</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H17" s="3">
@@ -1857,7 +1896,7 @@
       <c r="F18" t="s">
         <v>41</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="6" t="s">
         <v>35</v>
       </c>
       <c r="H18" s="3">
@@ -1904,7 +1943,7 @@
       <c r="F19" t="s">
         <v>56</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H19" s="3">
@@ -1957,7 +1996,7 @@
       <c r="F20" t="s">
         <v>56</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H20" s="3">
@@ -2010,7 +2049,7 @@
       <c r="F21" t="s">
         <v>45</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H21" s="3">
@@ -2060,7 +2099,7 @@
       <c r="F22" t="s">
         <v>34</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H22" s="3">
@@ -2113,7 +2152,7 @@
       <c r="F23" t="s">
         <v>45</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="6" t="s">
         <v>35</v>
       </c>
       <c r="H23" s="3">
@@ -2160,7 +2199,7 @@
       <c r="F24" t="s">
         <v>62</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="6" t="s">
         <v>35</v>
       </c>
       <c r="H24" s="3">
@@ -2207,7 +2246,7 @@
       <c r="F25" t="s">
         <v>41</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H25" s="3">
@@ -2257,7 +2296,7 @@
       <c r="F26" t="s">
         <v>34</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H26" s="3">
@@ -2307,7 +2346,7 @@
       <c r="F27" t="s">
         <v>41</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H27" s="3">
@@ -2360,7 +2399,7 @@
       <c r="F28" t="s">
         <v>45</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G28" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H28" s="3">
@@ -2413,7 +2452,7 @@
       <c r="F29" t="s">
         <v>45</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G29" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H29" s="3">
@@ -2463,7 +2502,7 @@
       <c r="F30" t="s">
         <v>41</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H30" s="3">
@@ -2513,7 +2552,7 @@
       <c r="F31" t="s">
         <v>62</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" s="6" t="s">
         <v>35</v>
       </c>
       <c r="H31" s="3">
@@ -2560,7 +2599,7 @@
       <c r="F32" t="s">
         <v>41</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H32" s="3">
@@ -2610,7 +2649,7 @@
       <c r="F33" t="s">
         <v>41</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H33" s="3">
@@ -2663,7 +2702,7 @@
       <c r="F34" t="s">
         <v>41</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G34" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H34" s="3">
@@ -2710,7 +2749,7 @@
       <c r="F35" t="s">
         <v>45</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H35" s="3">
@@ -2757,7 +2796,7 @@
       <c r="F36" t="s">
         <v>41</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G36" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H36" s="3">
@@ -2810,7 +2849,7 @@
       <c r="F37" t="s">
         <v>62</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H37" s="3">
@@ -2863,7 +2902,7 @@
       <c r="F38" t="s">
         <v>100</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H38" s="3">
@@ -2913,7 +2952,7 @@
       <c r="F39" t="s">
         <v>62</v>
       </c>
-      <c r="G39" t="s">
+      <c r="G39" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H39" s="3">
@@ -2966,7 +3005,7 @@
       <c r="F40" t="s">
         <v>34</v>
       </c>
-      <c r="G40" t="s">
+      <c r="G40" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H40" s="3">
@@ -3019,7 +3058,7 @@
       <c r="F41" t="s">
         <v>100</v>
       </c>
-      <c r="G41" t="s">
+      <c r="G41" s="6" t="s">
         <v>42</v>
       </c>
       <c r="H41" s="3">
@@ -3072,7 +3111,7 @@
       <c r="F42" t="s">
         <v>56</v>
       </c>
-      <c r="G42" t="s">
+      <c r="G42" s="6" t="s">
         <v>38</v>
       </c>
       <c r="H42" s="3">
@@ -6830,6 +6869,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="8.7265625" style="6"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -6838,7 +6880,7 @@
       <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D1" t="s">
@@ -6855,8 +6897,8 @@
       <c r="B2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="4">
-        <v>46023</v>
+      <c r="C2" s="6" t="s">
+        <v>158</v>
       </c>
       <c r="D2" t="s">
         <v>25</v>
@@ -6872,8 +6914,8 @@
       <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="4">
-        <v>46266</v>
+      <c r="C3" s="6" t="s">
+        <v>159</v>
       </c>
       <c r="D3" t="s">
         <v>26</v>
@@ -6886,8 +6928,8 @@
       <c r="A4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="4">
-        <v>46388</v>
+      <c r="C4" s="6" t="s">
+        <v>42</v>
       </c>
       <c r="E4" t="s">
         <v>151</v>
@@ -6897,8 +6939,8 @@
       <c r="A5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="4">
-        <v>46631</v>
+      <c r="C5" s="6" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -6930,7 +6972,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>28</v>
       </c>
     </row>
@@ -6940,35 +6982,35 @@
         <v>12 overdue, 4 due this week</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -6986,7 +7028,7 @@
       </c>
       <c r="D4" t="str">
         <f ca="1">IFERROR(INDEX(APPLICANTS!D:D,MATCH($A4,APPLICANTS!$P:$P,0))&amp;"","")</f>
-        <v/>
+        <v>Abuja</v>
       </c>
       <c r="E4" t="str">
         <f ca="1">IFERROR(INDEX(APPLICANTS!I:I,MATCH($A4,APPLICANTS!$P:$P,0))&amp;"","")</f>
@@ -7010,7 +7052,7 @@
       </c>
       <c r="J4" t="str">
         <f ca="1">IFERROR(INDEX(APPLICANTS!O:O,MATCH($A4,APPLICANTS!$P:$P,0))&amp;"","")</f>
-        <v/>
+        <v>Advisor 1</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>